<commit_message>
Got rid of of old comments from 'DECONSTRUCTOR'. Try to diff this commit and previous to see.
</commit_message>
<xml_diff>
--- a/Data/Edgecases.xlsx
+++ b/Data/Edgecases.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72844556-05E8-234B-B8E5-FD7854FB5203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{DF2B0E2F-E263-AF44-9DF2-4F2A0CA96ABD}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18900" xr2:uid="{DF2B0E2F-E263-AF44-9DF2-4F2A0CA96ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Started dev for 2 flush edgecase
</commit_message>
<xml_diff>
--- a/Data/Edgecases.xlsx
+++ b/Data/Edgecases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Malcolm/Documents/GitHub/Fantasyland/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72844556-05E8-234B-B8E5-FD7854FB5203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0BC953-D9FE-E248-8CB8-84439697A841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18900" xr2:uid="{DF2B0E2F-E263-AF44-9DF2-4F2A0CA96ABD}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Name</t>
   </si>
@@ -191,6 +191,12 @@
   </si>
   <si>
     <t>4, 5, 6, 7, 8, 9 straight where 5, 6, 7, 8, are duplicates and 7 is a triple. Got pair of Aces. Got Fantasy</t>
+  </si>
+  <si>
+    <t>16_Double_Flush_Dragon_Hardcode</t>
+  </si>
+  <si>
+    <t>[('2', 'Diamonds'), ('3', 'Diamonds'), ('4', 'Diamonds'), ('5', 'Clubs'), ('6', 'Clubs'), ('7', 'Hearts'), ('8', 'Hearts'), ('9', 'Diamonds'), ('10', 'Clubs'), ('J', 'Diamonds'),  ('Q', 'Clubs'), ('K', 'Diamonds'), ('A', 'Clubs')]</t>
   </si>
 </sst>
 </file>
@@ -546,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF0DCDF-CA70-BE49-A1E2-B9B130C8C33E}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.5" customWidth="1"/>
@@ -741,6 +747,14 @@
         <v>50</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
New commit in dev
</commit_message>
<xml_diff>
--- a/Data/Edgecases.xlsx
+++ b/Data/Edgecases.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Malcolm/Documents/GitHub/Fantasyland/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D0BC953-D9FE-E248-8CB8-84439697A841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3257113-EF2C-5B47-9B43-F5E009C9BB61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18900" xr2:uid="{DF2B0E2F-E263-AF44-9DF2-4F2A0CA96ABD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
   <si>
     <t>Name</t>
   </si>
@@ -197,6 +198,42 @@
   </si>
   <si>
     <t>[('2', 'Diamonds'), ('3', 'Diamonds'), ('4', 'Diamonds'), ('5', 'Clubs'), ('6', 'Clubs'), ('7', 'Hearts'), ('8', 'Hearts'), ('9', 'Diamonds'), ('10', 'Clubs'), ('J', 'Diamonds'),  ('Q', 'Clubs'), ('K', 'Diamonds'), ('A', 'Clubs')]</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Spades</t>
+  </si>
+  <si>
+    <t>Hearts</t>
+  </si>
+  <si>
+    <t>Clubs</t>
+  </si>
+  <si>
+    <t>Diamonds</t>
+  </si>
+  <si>
+    <t>17_2Flush_no_straight</t>
+  </si>
+  <si>
+    <t>[('2', 'Hearts'), ('2', 'Clubs'), ('4', 'Hearts'), ('4', 'Clubs'),  ('5', 'Hearts'), ('5', 'Diamonds'), ('5', 'Clubs'), ('9', 'Spades'), ('10', 'Hearts'), ('10', 'Clubs'),  ('K', 'Hearts'),  ('K', 'Clubs'), ('A', 'Spades')]</t>
+  </si>
+  <si>
+    <t>[('3', 'Diamonds'), ('4', 'Spades'), ('4', 'Clubs'), ('5', 'Spades'), ('5', 'Hearts'), ('6', 'Clubs'), ('7', 'Diamonds'), ('8', 'Spades'), ('10', 'Spades'), ('10', 'Hearts'), ('10', 'Clubs'), ('Q', 'Spades'), ('K', 'Spades')]</t>
+  </si>
+  <si>
+    <t>18_Case1</t>
   </si>
 </sst>
 </file>
@@ -212,12 +249,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -232,12 +275,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFF0DCDF-CA70-BE49-A1E2-B9B130C8C33E}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.5" customWidth="1"/>
@@ -755,6 +799,228 @@
         <v>52</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFF239B1-C1F5-BF4A-9BE6-9F0ACBF9849D}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>7</v>
+      </c>
+      <c r="C8" s="3">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>